<commit_message>
Accessibility sheet: keyboard walk-through evidence and three closed defects
2.1.1 / 2.1.2 / 2.4.3 / 2.4.7 / 2.4.11 reviewed on the strength of
scripts/browser/keyboard-walk.mjs (0 problems on production after
ce4c4c9); the aria-label comma bug, the cart-drawer focus loss and the
headless-session counting recorded as done.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
+++ b/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="15.75" customWidth="1" style="41" min="1" max="1"/>
@@ -893,301 +893,412 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Manual keyboard walk-through</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>2.1.1: Keyboard</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Automated with scripts/browser/keyboard-walk.mjs (Playwright, real key events): 0 problems on production after ce4c4c9. A human NVDA pass remains advisable but the keyboard model is proven.</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Focus visible + not obscured</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>2.4.7: Focus Visible</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>keyboard-walk.mjs checks outline/box-shadow on every stop and header overlap; 0 problems at 1280x800. Footer ring #D2AC55 = 7.5:1.</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Resize text 200% / text spacing</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>1.4.4: Resize Text</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Tab through home -&gt; PDP gallery -&gt; quantity -&gt; add to cart -&gt; cart drawer -&gt; checkout link on Chrome + NVDA. Confirm no trap in the drawer (2.1.2) and focus returns to the trigger on close.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>Set browser base font to 32 px and run the text-spacing bookmarklet on home, PDP, cart. CI covers reflow at 320 px but not font scaling.</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Dimension-diagram alt text</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>1.1.1: Non-text Content</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>The supplier diagrams (now image 2 on 18 products) carry alts that read the numbers; confirm each matches the copy's 'What you get' sizes after the 2026-09-18 image changes.</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Focus visible + not obscured</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2.4.7: Focus Visible</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Checkout is Shopify-hosted</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>3.3.1: Error Identification</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Verify the focus ring on the navy hero buttons and inside the cart drawer; confirm the sticky header never covers a focused element at 390 px (2.4.11).</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>checkout.puchica.ca is Shopify Checkout - forms, errors, autofill (1.3.5), redundant entry (3.3.7) are Shopify's surface. Record that scope boundary here; test once with a real address anyway.</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Heading before H1 in dialogs</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>1.3.1: Info and Relationships</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>Cart/Search/Menu dialogs put H3s before the page H1 in DOM order. Hidden until opened, so not a failure; consider aria-labelledby on the dialogs instead of headings.</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Resize text 200% / text spacing</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1.4.4: Resize Text</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Set browser base font to 32 px and run the text-spacing bookmarklet on home, PDP, cart. CI covers reflow at 320 px but not font scaling.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>PDP had no CI coverage</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>2.4.2: Page Titled</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>tests/browser/production.spec.js audited /products/travel-cable-organizer-case (deleted 2026-08-28) - a 404 - for three weeks. Now audits the globe PDP and /pages/about. Commit 76eb6b4.</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Dimension-diagram alt text</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1.1.1: Non-text Content</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>The supplier diagrams (now image 2 on 18 products) carry alts that read the numbers; confirm each matches the copy's 'What you get' sizes after the 2026-09-18 image changes.</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>About page title</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>2.4.2: Page Titled</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>'About Puchica | A focused Canadian travel shop' -&gt; 'A small Canadian lighting shop' in 4 locales. Commit 76eb6b4.</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Checkout is Shopify-hosted</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>3.3.1: Error Identification</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>checkout.puchica.ca is Shopify Checkout - forms, errors, autofill (1.3.5), redundant entry (3.3.7) are Shopify's surface. Record that scope boundary here; test once with a real address anyway.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Heading before H1 in dialogs</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1.3.1: Info and Relationships</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Cart/Search/Menu dialogs put H3s before the page H1 in DOM order. Hidden until opened, so not a failure; consider aria-labelledby on the dialogs instead of headings.</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Shipping H1 accessible name</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>1.3.2: Meaningful Sequence</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>'Shipping &amp;Delivery.' -&gt; 'Shipping &amp; Delivery.' (whitespace between spans). Commit 76eb6b4.</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>PDP had no CI coverage</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2.4.2: Page Titled</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>aria-label comma bug in t()</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>4.1.2: Name, Role, Value</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>tests/browser/production.spec.js audited /products/travel-cable-organizer-case (deleted 2026-08-28) - a 404 - for three weeks. Now audits the globe PDP and /pages/about. Commit 76eb6b4.</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>t() with params returned an array -&gt; React comma-joined every aria-label built with it (thumbnails, cards). Fixed in app/lib/t.js, 5e8af70.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>keyboard-walk.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Content</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>About page title</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2.4.2: Page Titled</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cart drawer Escape lost focus</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2.4.3: Focus Order</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>'About Puchica | A focused Canadian travel shop' -&gt; 'A small Canadian lighting shop' in 4 locales. Commit 76eb6b4.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Saved element was &lt;body&gt; because the add-to-cart form re-mounts while the cart fetch completes. Aside now returns focus to the drawer's own trigger via data-focus-return (5e8af70, ce4c4c9).</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>keyboard-walk.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Shipping H1 accessible name</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1.3.2: Meaningful Sequence</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Shopify sessions counted headless browsers</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>n/a (measurement)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>'Shipping &amp;Delivery.' -&gt; 'Shipping &amp; Delivery.' (whitespace between spans). Commit 76eb6b4.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Analytics.Provider canTrack now returns false for headless/bot UAs (da56b6e); CI Playwright runs no longer create sessions.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>app/root.jsx</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="41"/>
     <row r="22" ht="15.75" customHeight="1" s="41"/>
@@ -4091,7 +4202,7 @@
       </c>
       <c r="F44" s="25" t="inlineStr">
         <is>
-          <t>All controls are native &lt;a&gt;/&lt;button&gt;/&lt;input&gt;; gallery thumbnails are buttons. Manual keyboard walk-through of the PDP gallery and cart drawer is on the Task List - not yet done by a human.</t>
+          <t>All controls reachable and operable by keyboard; Enter on Add to cart opens the cart drawer, Escape closes it. scripts/browser/keyboard-walk.mjs on production 2026-09-18 04:50 (after ce4c4c9): home 44 stops, PDP 19 + cart drawer, /collections/all 72 stops; 0 problems. NVDA/VoiceOver pass by a human still recommended before ads.</t>
         </is>
       </c>
       <c r="G44" s="25" t="inlineStr">
@@ -4128,14 +4239,18 @@
         </is>
       </c>
       <c r="D45" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 2.1.2: No Keyboard Trap</t>
         </is>
       </c>
-      <c r="F45" s="25" t="n"/>
+      <c r="F45" s="25" t="inlineStr">
+        <is>
+          <t>No trap: Tab cycles inside the open cart drawer (Aside focus trap) and Escape releases it; page tab order wraps to body. scripts/browser/keyboard-walk.mjs on production 2026-09-18 04:50 (after ce4c4c9): home 44 stops, PDP 19 + cart drawer, /collections/all 72 stops; 0 problems.</t>
+        </is>
+      </c>
       <c r="G45" s="25" t="inlineStr">
         <is>
           <t>A</t>
@@ -4468,14 +4583,18 @@
         </is>
       </c>
       <c r="D53" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 2.4.11: Focus Not Obscured (Minimum) | WAI | W3C</t>
         </is>
       </c>
-      <c r="F53" s="25" t="n"/>
+      <c r="F53" s="25" t="inlineStr">
+        <is>
+          <t>No focused element sat under the sticky header at 1280x800; the skip link renders above it (z-index 9999). scripts/browser/keyboard-walk.mjs on production 2026-09-18 04:50 (after ce4c4c9): home 44 stops, PDP 19 + cart drawer, /collections/all 72 stops; 0 problems.</t>
+        </is>
+      </c>
       <c r="G53" s="25" t="inlineStr">
         <is>
           <t>AA</t>
@@ -4644,14 +4763,18 @@
         </is>
       </c>
       <c r="D57" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E57" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 2.4.3: Focus Order</t>
         </is>
       </c>
-      <c r="F57" s="25" t="n"/>
+      <c r="F57" s="25" t="inlineStr">
+        <is>
+          <t>Focus order follows the visual order (skip link, header, breadcrumb, chips, cards, footer). Escape from the cart drawer now returns focus to the Add to cart button (was &lt;body&gt; - fixed 5e8af70/ce4c4c9). scripts/browser/keyboard-walk.mjs on production 2026-09-18 04:50 (after ce4c4c9): home 44 stops, PDP 19 + cart drawer, /collections/all 72 stops; 0 problems.</t>
+        </is>
+      </c>
       <c r="G57" s="25" t="inlineStr">
         <is>
           <t>A</t>
@@ -5026,14 +5149,18 @@
         </is>
       </c>
       <c r="D66" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 2.4.7: Focus Visible</t>
         </is>
       </c>
-      <c r="F66" s="25" t="n"/>
+      <c r="F66" s="25" t="inlineStr">
+        <is>
+          <t>Every stop showed a visible indicator (clay outline on paper; light honey #D2AC55 in the footer). scripts/browser/keyboard-walk.mjs on production 2026-09-18 04:50 (after ce4c4c9): home 44 stops, PDP 19 + cart drawer, /collections/all 72 stops; 0 problems.</t>
+        </is>
+      </c>
       <c r="G66" s="25" t="inlineStr">
         <is>
           <t>AA</t>
@@ -6517,7 +6644,7 @@
       </c>
       <c r="F101" s="25" t="inlineStr">
         <is>
-          <t>No custom widgets outside native elements + dialogs. axe-core 4.x, WCAG 2.0/2.1/2.2 A+AA + best-practice, 7 routes (home, /collections/all, PDP globe, about, shipping, cart, search) at 1440 and 390 px, 2026-09-18: 0 violations at any impact. CI #153 also green (105 checks).</t>
+          <t>No custom widgets outside native elements + dialogs. axe 0 violations. FIXED 2026-09-18: t() with params returned an array, so aria-label read "View image ,1, of ,2," and "View ,&lt;title&gt;," on every thumbnail and card; t() now returns a string when every value is text (commit 5e8af70).</t>
         </is>
       </c>
       <c r="G101" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Product schema: inline return policy + shipping details, Organization on PDP
Schema audit of all 20 product pages (work/schema-audit.mjs, 2026-09-19):
every Offer's hasMerchantReturnPolicy was an @id pointer to a node that
only the homepage emits, so on the PDP itself Google saw no return
policy; no Offer carried shippingDetails; no PDP carried the
Organization. Merchant listings / rich results need all three.

seo.js now exports merchantReturnPolicyJsonLd() and
shippingDetailsJsonLd() (Canada only, free, 1-3 day handling, 10-21 day
transit = the FAQ's "two to three weeks"); the Organization uses the
same policy builder; the product Offer inlines both and the PDP emits
the Organization script. Accessibility sheet rows from 18 Sep committed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
+++ b/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="15.75" customWidth="1" style="41" min="1" max="1"/>
@@ -1190,113 +1190,298 @@
       <c r="G11" s="0" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>aria-label comma bug in t()</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>4.1.2: Name, Role, Value</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="0" t="inlineStr">
         <is>
           <t>t() with params returned an array -&gt; React comma-joined every aria-label built with it (thumbnails, cards). Fixed in app/lib/t.js, 5e8af70.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t>keyboard-walk.mjs</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Cart drawer Escape lost focus</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>2.4.3: Focus Order</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>Saved element was &lt;body&gt; because the add-to-cart form re-mounts while the cart fetch completes. Aside now returns focus to the drawer's own trigger via data-focus-return (5e8af70, ce4c4c9).</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t>keyboard-walk.mjs</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Shopify sessions counted headless browsers</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>n/a (measurement)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="0" t="inlineStr">
         <is>
           <t>Analytics.Provider canTrack now returns false for headless/bot UAs (da56b6e); CI Playwright runs no longer create sessions.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>app/root.jsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Canada-only market close</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>n/a (content accuracy)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>U.S market set to draft + US shipping zone removed 2026-09-18; every locale's FAQ/contact/terms copy, the return-policy schema and the brand description now say Canada only (7e68668). Screen-reader users no longer hear a market/currency that checkout will refuse.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>curl + metadata-health, 4 locales</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PDP &lt;title&gt; carries the brand</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.4.2: Page Titled</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SEO titles written without 'Puchica' made every product tab title brand-less; route now appends ' – Puchica' unless the stored title already names it (8c9c13e). metadata-health 116/116.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>npm run metadata-health</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cart line thumbnails were blank</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.1.1: Non-text Content</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>15/20 variants had no image bound, so /cart, the drawer and checkout showed an empty box beside the product name. Variants rebound to their lifestyle heroes; storefront falls back to product.featuredImage (354c90b). Alt text = variant alt or product title.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>checkout walk-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Self-hosted fonts, no layout shift</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2.2.2 / CWV</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>fonts.googleapis.com stylesheet was render-blocking (~0.9 s LCP on mobile). Fraunces + Instrument Sans now served from /fonts with font-display: swap; CLS stayed 0–0.03 (96352b7).</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Lighthouse work/lighthouse/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Post-change production audit</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>multiple</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-09-18 evening after the Canada-only close: Playwright 105/105, axe 0 violations (7 routes × 2 viewports), keyboard walk 0 problems, metadata 116/116, links 152/152.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>scripts/browser/*, npx playwright test</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Accessibility sheet: 19 Sep loop rows; organic pack captions
Sheet: live regions and 200% zoom items closed with evidence; rows added
for Product schema, home hero LCP, facts-row locale test and the
add-to-cart probe; one new low item for the 1.4.12 text-spacing pass.

work/organic/2026-09-19/README.md: Instagram, Pinterest and
Marketplace/Kijiji captions, alt text and PDP links for the globe, gourd,
slatted lantern and rattan cone. Numbers copied from the live PDPs; no
discounts.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
+++ b/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="15.75" customWidth="1" style="41" min="1" max="1"/>
@@ -858,7 +858,7 @@
     <row r="2" ht="22.5" customHeight="1" s="41">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
@@ -878,17 +878,17 @@
       </c>
       <c r="E2" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F2" s="31" t="inlineStr">
         <is>
-          <t>/collections/all renders ~18 role=status nodes (one per product card) and the PDP ~8. Screen readers announce each. Move add-to-cart feedback to a single page-level live region.</t>
+          <t>2026-09-19: one polite live region for the whole page (app/components/LiveAnnouncer.jsx, mounted in PageLayout). AddToCartButton calls announce(); the per-card role=status spans are gone. /collections/all: 22 regions -&gt; 1. axe 0, keyboard walk 0.</t>
         </is>
       </c>
       <c r="G2" s="20" t="inlineStr">
         <is>
-          <t>scripts/browser/axe-full-sweep.mjs landmark snapshot 2026-09-18</t>
+          <t>LiveAnnouncer.jsx; scripts/browser/axe-full-sweep.mjs</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
@@ -981,15 +981,19 @@
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>Set browser base font to 32 px and run the text-spacing bookmarklet on home, PDP, cart. CI covers reflow at 320 px but not font scaling.</t>
-        </is>
-      </c>
-      <c r="G5" s="0" t="inlineStr"/>
+          <t>2026-09-19: scripts/browser/zoom-reflow.mjs runs the 5 production routes at 320px wide and at CSS zoom 2 (200%), flags any box clipped past the viewport or overlapping text: 0 problems. Newsletter honeypot was the one hit (left:-10000px) and is now clipped in place. Text-spacing bookmarklet (1.4.12) still a manual item.</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>scripts/browser/zoom-reflow.mjs</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -1301,194 +1305,375 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Canada-only market close</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>n/a (content accuracy)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="0" t="inlineStr">
         <is>
           <t>U.S market set to draft + US shipping zone removed 2026-09-18; every locale's FAQ/contact/terms copy, the return-policy schema and the brand description now say Canada only (7e68668). Screen-reader users no longer hear a market/currency that checkout will refuse.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="0" t="inlineStr">
         <is>
           <t>curl + metadata-health, 4 locales</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>PDP &lt;title&gt; carries the brand</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>2.4.2: Page Titled</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="0" t="inlineStr">
         <is>
           <t>SEO titles written without 'Puchica' made every product tab title brand-less; route now appends ' – Puchica' unless the stored title already names it (8c9c13e). metadata-health 116/116.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="0" t="inlineStr">
         <is>
           <t>npm run metadata-health</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Cart line thumbnails were blank</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>1.1.1: Non-text Content</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="0" t="inlineStr">
         <is>
           <t>15/20 variants had no image bound, so /cart, the drawer and checkout showed an empty box beside the product name. Variants rebound to their lifestyle heroes; storefront falls back to product.featuredImage (354c90b). Alt text = variant alt or product title.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="0" t="inlineStr">
         <is>
           <t>checkout walk-through</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Self-hosted fonts, no layout shift</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>2.2.2 / CWV</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="0" t="inlineStr">
         <is>
           <t>fonts.googleapis.com stylesheet was render-blocking (~0.9 s LCP on mobile). Fraunces + Instrument Sans now served from /fonts with font-display: swap; CLS stayed 0–0.03 (96352b7).</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="0" t="inlineStr">
         <is>
           <t>Lighthouse work/lighthouse/README.md</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Post-change production audit</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>multiple</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="0" t="inlineStr">
         <is>
           <t>2026-09-18 evening after the Canada-only close: Playwright 105/105, axe 0 violations (7 routes × 2 viewports), keyboard walk 0 problems, metadata 116/116, links 152/152.</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t>scripts/browser/*, npx playwright test</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="41"/>
-    <row r="22" ht="15.75" customHeight="1" s="41"/>
-    <row r="23" ht="15.75" customHeight="1" s="41"/>
-    <row r="24" ht="15.75" customHeight="1" s="41"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Product structured data complete</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>n/a (SEO / findability)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-09-19: all 20 PDPs carry Product JSON-LD with name, image, description, sku, brand, offers (CAD price, availability, url), OfferShippingDetails (CA, free, 1-3 d handling, 10-21 d transit) and MerchantReturnPolicy (CA, 30 d). Organization + BreadcrumbList on every PDP. work/schema-audit.mjs: 20/20 pass; metadata-health green.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>app/lib/seo.js; work/schema-audit.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="41">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Home hero LCP</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2.2.2 / CWV</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-09-19: hero is a &lt;picture&gt; with a 3:4 CDN crop for phones (412/640w) and square crops for desktop, preloaded via meta() link descriptors with fetchpriority=high. Lighthouse devtools throttling: home LCP 4.1 s -&gt; 3.24 s, CLS 0; collection 7.9 -&gt; 2.7 s; PDP 2.8 s.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>app/lib/hero-image.js; work/lighthouse/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1" s="41">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Facts row complete in all 4 locales</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1.3.1: Info and Relationships</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-09-19: every approved handle x locale shows &gt;=3 facts; sconces show 4 (Size, Backplate/Mount, Fitting, Bulb). Spanish casquillo and the EN Mount label were unmatched before. Title cm vs Size-fact differences are deliberate rounding (14.5-&gt;15 etc.).</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>tests/product-facts-locales.test.js; work/copy-audit.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="41">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Add-to-cart first click</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>n/a (measurement)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-09-19: Playwright probe, 5 PDPs x 4 runs, click immediately after load and after networkidle: 40/40 increments the cart count on the first click. No pre-hydration bug; nothing changed.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>work/atc-probe.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="41">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Text spacing bookmarklet (1.4.12)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.4.12: Text Spacing</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Apply the WCAG text-spacing overrides (line-height 1.5, paragraph 2em, letter 0.12em, word 0.16em) on the 5 routes and look for clipping. Could be folded into zoom-reflow.mjs as a third pass.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>scripts/browser/zoom-reflow.mjs</t>
+        </is>
+      </c>
+    </row>
     <row r="25" ht="15.75" customHeight="1" s="41"/>
     <row r="26" ht="15.75" customHeight="1" s="41"/>
     <row r="27" ht="15.75" customHeight="1" s="41"/>
@@ -3703,7 +3888,7 @@
       </c>
       <c r="F28" s="25" t="inlineStr">
         <is>
-          <t>CI probe findOverflow at 320 x 800 on 5 routes: no horizontal scroll, run #153. 400% zoom equivalent.</t>
+          <t>CI probe findOverflow at 320 x 800 on 5 routes: no horizontal scroll, run #153. 400% zoom equivalent. Plus scripts/browser/zoom-reflow.mjs at 320px and 200% zoom: 0 problems (2026-09-19).</t>
         </is>
       </c>
       <c r="G28" s="25" t="inlineStr">
@@ -4210,14 +4395,18 @@
         </is>
       </c>
       <c r="D40" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 1.4.4: Resize Text</t>
         </is>
       </c>
-      <c r="F40" s="25" t="n"/>
+      <c r="F40" s="25" t="inlineStr">
+        <is>
+          <t>zoom-reflow.mjs at CSS zoom 2 on 5 routes: no clipped or overlapping text (2026-09-19).</t>
+        </is>
+      </c>
       <c r="G40" s="25" t="inlineStr">
         <is>
           <t>AA</t>
@@ -6917,7 +7106,7 @@
       </c>
       <c r="F103" s="25" t="inlineStr">
         <is>
-          <t>Add-to-cart feedback and cart recovery banner are role=status. OPEN: /collections/all exposes ~18 role=status regions (one per card) and the PDP ~8 - noisy for screen readers; consolidate to one live region per page (Task List).</t>
+          <t>Single polite live region (LiveAnnouncer) announces add-to-cart adding/added/failed; per-card status spans removed (2026-09-19).</t>
         </is>
       </c>
       <c r="G103" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Lockfile: add @emnapi entries npm ci needs; sheet rows for NVDA + Quebec
npm ci on CI (Node 22) refused the lock written on Windows: @emnapi/core
and @emnapi/runtime were missing. Regenerated with --package-lock-only
under Node 22.19 and verified npm ci passes.

Accessibility sheet: scripted NVDA walk row (done) and Quebec cookie
consent row (done).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
+++ b/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="15.75" customWidth="1" style="41" min="1" max="1"/>
@@ -1490,192 +1490,264 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Product structured data complete</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>n/a (SEO / findability)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="0" t="inlineStr">
         <is>
           <t>2026-09-19: all 20 PDPs carry Product JSON-LD with name, image, description, sku, brand, offers (CAD price, availability, url), OfferShippingDetails (CA, free, 1-3 d handling, 10-21 d transit) and MerchantReturnPolicy (CA, 30 d). Organization + BreadcrumbList on every PDP. work/schema-audit.mjs: 20/20 pass; metadata-health green.</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t>app/lib/seo.js; work/schema-audit.mjs</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="41">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Home hero LCP</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>2.2.2 / CWV</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="0" t="inlineStr">
         <is>
           <t>2026-09-19: hero is a &lt;picture&gt; with a 3:4 CDN crop for phones (412/640w) and square crops for desktop, preloaded via meta() link descriptors with fetchpriority=high. Lighthouse devtools throttling: home LCP 4.1 s -&gt; 3.24 s, CLS 0; collection 7.9 -&gt; 2.7 s; PDP 2.8 s.</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t>app/lib/hero-image.js; work/lighthouse/README.md</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="41">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Facts row complete in all 4 locales</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>1.3.1: Info and Relationships</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="0" t="inlineStr">
         <is>
           <t>2026-09-19: every approved handle x locale shows &gt;=3 facts; sconces show 4 (Size, Backplate/Mount, Fitting, Bulb). Spanish casquillo and the EN Mount label were unmatched before. Title cm vs Size-fact differences are deliberate rounding (14.5-&gt;15 etc.).</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t>tests/product-facts-locales.test.js; work/copy-audit.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="41">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>Add-to-cart first click</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>n/a (measurement)</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="0" t="inlineStr">
         <is>
           <t>2026-09-19: Playwright probe, 5 PDPs x 4 runs, click immediately after load and after networkidle: 40/40 increments the cart count on the first click. No pre-hydration bug; nothing changed.</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t>work/atc-probe.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="41">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Text spacing bookmarklet (1.4.12)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>1.4.12: Text Spacing</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="0" t="inlineStr">
         <is>
           <t>Apply the WCAG text-spacing overrides (line-height 1.5, paragraph 2em, letter 0.12em, word 0.16em) on the 5 routes and look for clipping. Could be folded into zoom-reflow.mjs as a third pass.</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t>scripts/browser/zoom-reflow.mjs</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="41"/>
-    <row r="26" ht="15.75" customHeight="1" s="41"/>
+    <row r="25" ht="15.75" customHeight="1" s="41">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Screen-reader walk (NVDA, scripted)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>4.1.2 / 4.1.3 / 1.3.1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-09-20: npm run nvda-walk drives a real NVDA (guidepup) over the PDP, the add-to-cart flow and the footer form; transcripts in work/nvda/2026-09-20. Reading order, price-after-name, button roles, the live-region announcement (Adding… / Added), the cart dialog and the form labels all read correctly. Finding fixed in 9efabab: the wordmark ¡púchica! was read as "inverted exclamation point púchica!" — links now have aria-label Puchica — Home and the announcer drops inverted punctuation. Human listen-through of the transcript still worthwhile; it is a 5-minute read.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>scripts/browser/nvda-walk.mjs; work/nvda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="41">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Quebec cookie consent (Law 25)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>n/a (privacy)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-09-19: Shopify Customer privacy → cookie banner regions set manually: Quebec (CAQC) consentRequired=true plus the EU/UK recommended set; rest of Canada unchanged. Verified via consentPolicy query. Hydrogen banner already wired (withPrivacyBanner). Needs a Quebec visitor to confirm it renders.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Shopify admin; consentPolicy API</t>
+        </is>
+      </c>
+    </row>
     <row r="27" ht="15.75" customHeight="1" s="41"/>
     <row r="28" ht="15.75" customHeight="1" s="41"/>
     <row r="29" ht="15.75" customHeight="1" s="41"/>
@@ -7018,7 +7090,7 @@
       </c>
       <c r="F101" s="25" t="inlineStr">
         <is>
-          <t>No custom widgets outside native elements + dialogs. axe 0 violations. FIXED 2026-09-18: t() with params returned an array, so aria-label read "View image ,1, of ,2," and "View ,&lt;title&gt;," on every thumbnail and card; t() now returns a string when every value is text (commit 5e8af70).</t>
+          <t>No custom widgets outside native elements + dialogs. axe 0 violations. FIXED 2026-09-18: t() with params returned an array, so aria-label read "View image ,1, of ,2," and "View ,&lt;title&gt;," on every thumbnail and card; t() now returns a string when every value is text (commit 5e8af70). NVDA walk 2026-09-20: roles and names spoken as expected (heading level 1, button, dialog, edit required); wordmark links given a plain accessible name.</t>
         </is>
       </c>
       <c r="G101" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Accessibility sheet: text-spacing pass done, home LCP row
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
+++ b/docs/accessibility/Puchica-Accessibility-Sheet-2026-09-18.xlsx
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col width="15.75" customWidth="1" style="41" min="1" max="1"/>
@@ -1640,7 +1640,7 @@
     <row r="24" ht="15.75" customHeight="1" s="41">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -1660,12 +1660,12 @@
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>
-          <t>Apply the WCAG text-spacing overrides (line-height 1.5, paragraph 2em, letter 0.12em, word 0.16em) on the 5 routes and look for clipping. Could be folded into zoom-reflow.mjs as a third pass.</t>
+          <t>2026-09-20: zoom-reflow.mjs has a third pass at 390px with the 1.4.12 overrides (line-height 1.5, paragraph 2em, letter 0.12em, word 0.16em): 0 problems on the 5 routes. The one hit was a link inside the collapsed Shipping &amp; Returns disclosure whose clipped box landed on the footer logo; the probe now clips control boxes by overflow ancestors.</t>
         </is>
       </c>
       <c r="G24" s="0" t="inlineStr">
@@ -1675,80 +1675,116 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="41">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Screen-reader walk (NVDA, scripted)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>4.1.2 / 4.1.3 / 1.3.1</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="0" t="inlineStr">
         <is>
           <t>2026-09-20: npm run nvda-walk drives a real NVDA (guidepup) over the PDP, the add-to-cart flow and the footer form; transcripts in work/nvda/2026-09-20. Reading order, price-after-name, button roles, the live-region announcement (Adding… / Added), the cart dialog and the form labels all read correctly. Finding fixed in 9efabab: the wordmark ¡púchica! was read as "inverted exclamation point púchica!" — links now have aria-label Puchica — Home and the announcer drops inverted punctuation. Human listen-through of the transcript still worthwhile; it is a 5-minute read.</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="0" t="inlineStr">
         <is>
           <t>scripts/browser/nvda-walk.mjs; work/nvda/</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="41">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>Dev</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Quebec cookie consent (Law 25)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>n/a (privacy)</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="0" t="inlineStr">
         <is>
           <t>2026-09-19: Shopify Customer privacy → cookie banner regions set manually: Quebec (CAQC) consentRequired=true plus the EU/UK recommended set; rest of Canada unchanged. Verified via consentPolicy query. Hydrogen banner already wired (withPrivacyBanner). Needs a Quebec visitor to confirm it renders.</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="0" t="inlineStr">
         <is>
           <t>Shopify admin; consentPolicy API</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="41"/>
+    <row r="27" ht="15.75" customHeight="1" s="41">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Home LCP under 3 s</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2.2.2 / CWV</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-09-20: font preloads removed (they competed with the hero image on a throttled phone). Lighthouse devtools throttling: LCP 3.2 s -&gt; 2.78 s, CLS 0, perf 78. font-display: swap keeps text painting immediately.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>work/lighthouse/README.md</t>
+        </is>
+      </c>
+    </row>
     <row r="28" ht="15.75" customHeight="1" s="41"/>
     <row r="29" ht="15.75" customHeight="1" s="41"/>
     <row r="30" ht="15.75" customHeight="1" s="41"/>
@@ -4085,14 +4121,18 @@
         </is>
       </c>
       <c r="D31" s="26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" s="28" t="inlineStr">
         <is>
           <t>Understanding Success Criterion 1.4.12: Text Spacing</t>
         </is>
       </c>
-      <c r="F31" s="25" t="n"/>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>zoom-reflow.mjs text-spacing pass, 5 routes at 390px: no clipped or overlapping content (2026-09-20).</t>
+        </is>
+      </c>
       <c r="G31" s="25" t="inlineStr">
         <is>
           <t>AA</t>

</xml_diff>